<commit_message>
feat: perfiles enriquecidos de conferencistas con vista de detalle y fotos
Cada card ahora abre un modal con formacion academica, trayectoria y foto
de perfil, todo leido en vivo desde nuevas columnas de la hoja Base de
Datos del Excel (titulo_profesional, formacion_academica,
trayectoria_destacada). Las fotos y el aro floral institucional, extraidos
de los perfiles en PowerPoint de cada conferencista, se resuelven por
convencion de archivo a partir del slug ya existente, sin agregar columnas
para eso. Se quita el truncado de texto en las cards.

De paso corrige un bug real de posicionamiento del componente Dialog
compartido bajo el modo movil de escritorio forzado: WebKit resuelve mal
los porcentajes de alto para elementos position:fixed en ese contexto,
dejando cualquier modal fuera del area visible. Se cambia a position:
absolute con centrado calculado en JS a partir de valores de viewport
confiables.
</commit_message>
<xml_diff>
--- a/portal-web/data/source-conferencistas/Participacion jornadas.xlsx
+++ b/portal-web/data/source-conferencistas/Participacion jornadas.xlsx
@@ -1702,9 +1702,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3B845049-F7AD-49C2-9B60-1D64B5A6D719}" name="tblParticipantesWeb" displayName="tblParticipantesWeb" ref="A1:AB13" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
-  <autoFilter ref="A1:AB13" xr:uid="{3B845049-F7AD-49C2-9B60-1D64B5A6D719}"/>
-  <tableColumns count="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3B845049-F7AD-49C2-9B60-1D64B5A6D719}" name="tblParticipantesWeb" displayName="tblParticipantesWeb" ref="A1:AE13" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+  <autoFilter ref="A1:AE13" xr:uid="{3B845049-F7AD-49C2-9B60-1D64B5A6D719}"/>
+  <tableColumns count="31">
     <tableColumn id="1" xr3:uid="{8F8C6840-79E6-4189-B5B0-93B41F28D108}" name="id_registro" dataDxfId="29"/>
     <tableColumn id="2" xr3:uid="{2F7D01C2-8836-4ED3-BE58-70A8E4DA99D6}" name="id_jornada" dataDxfId="28"/>
     <tableColumn id="3" xr3:uid="{B768C9DF-286B-40BA-A793-B5EA5B84F756}" name="jornada" dataDxfId="22"/>
@@ -1733,6 +1733,9 @@
     <tableColumn id="26" xr3:uid="{CA9921E3-7A4D-4450-939F-5BE3735AC9CD}" name="orden_card" dataDxfId="27"/>
     <tableColumn id="27" xr3:uid="{4A23AD6E-7472-4DF3-B60A-30E179BA21B9}" name="tipo_card" dataDxfId="26"/>
     <tableColumn id="28" xr3:uid="{23825030-4431-44B5-AF5D-B3D5A4129CD3}" name="publicar" dataDxfId="25"/>
+    <tableColumn id="29" xr3:uid="{A1B2C3D4-0001-4E00-8000-000000000001}" name="titulo_profesional"/>
+    <tableColumn id="30" xr3:uid="{A1B2C3D4-0001-4E00-8000-000000000002}" name="formacion_academica"/>
+    <tableColumn id="31" xr3:uid="{A1B2C3D4-0001-4E00-8000-000000000003}" name="trayectoria_destacada"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2471,7 +2474,7 @@
   <sheetPr>
     <tabColor rgb="FF4472C4"/>
   </sheetPr>
-  <dimension ref="A1:AB13"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.08984375" bestFit="1" customWidth="1"/>
@@ -2502,9 +2505,12 @@
     <col min="26" max="26" width="15" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="13.36328125" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="34" customWidth="1"/>
+    <col min="30" max="30" width="55" customWidth="1"/>
+    <col min="31" max="31" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:31" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="64" t="s">
         <v>58</v>
       </c>
@@ -2589,8 +2595,23 @@
       <c r="AB1" s="65" t="s">
         <v>155</v>
       </c>
+      <c r="AC1" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">titulo_profesional</t>
+        </is>
+      </c>
+      <c r="AD1" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">formacion_academica</t>
+        </is>
+      </c>
+      <c r="AE1" s="68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">trayectoria_destacada</t>
+        </is>
+      </c>
     </row>
-    <row r="2" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="64">
         <v>1</v>
       </c>
@@ -2663,8 +2684,11 @@
       <c r="AB2" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC2" s="69"/>
+      <c r="AD2" s="69"/>
+      <c r="AE2" s="69"/>
     </row>
-    <row r="3" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="64">
         <v>2</v>
       </c>
@@ -2737,8 +2761,11 @@
       <c r="AB3" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC3" s="69"/>
+      <c r="AD3" s="69"/>
+      <c r="AE3" s="69"/>
     </row>
-    <row r="4" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A4" s="64">
         <v>3</v>
       </c>
@@ -2817,8 +2844,28 @@
       <c r="AB4" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC4" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exrectora de la Universidad Colegio Mayor de Cundinamarca</t>
+        </is>
+      </c>
+      <c r="AD4" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doctora en Administración (México)
+MBA
+Magíster en Docencia Universitaria</t>
+        </is>
+      </c>
+      <c r="AE4" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exrectora de la Universidad Colegio Mayor de Cundinamarca y actual miembro del Consejo Superior Universitario
+Más de 27 años de experiencia en educación superior, liderazgo estratégico y gestión del talento humano
+Experta en diseño curricular, autoevaluación, acreditación de alta calidad y virtualización académica (COIL y clases espejo)
+Investigadora Junior (Colciencias 2024), vinculada a grupos A1 y con trayectoria como conferencista y consultora</t>
+        </is>
+      </c>
     </row>
-    <row r="5" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="64">
         <v>4</v>
       </c>
@@ -2897,8 +2944,28 @@
       <c r="AB5" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC5" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Docente permanente, Universidade Federal do Delta do Parnaíba (Brasil)</t>
+        </is>
+      </c>
+      <c r="AD5" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doctora en Psicología de la Educación, Universidad de Barcelona
+Máster en Psicología de la Educación y Psicología Social
+Licenciada en Psicología</t>
+        </is>
+      </c>
+      <c r="AE5" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ex Vicerrectora Académica, investigadora y líder de proyectos en educación superior, innovación educativa y tecnologías digitales aplicadas al aprendizaje
+Más de 20 años de experiencia en docencia, gestión académica e investigación en psicología y educación
+Liderazgo académico, producción científica y coordinación de grupos de investigación con reconocimiento nacional e internacional
+Reconocimientos: Premio Mujer Destacada 2024 y Doctor Honoris Causa 2023</t>
+        </is>
+      </c>
     </row>
-    <row r="6" spans="1:28" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="64">
         <v>5</v>
       </c>
@@ -2981,8 +3048,27 @@
       <c r="AB6" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC6" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Viceministro de Educación Superior de Colombia</t>
+        </is>
+      </c>
+      <c r="AD6" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Licenciado en Ciencias Sociales
+Magíster en Investigación Social Interdisciplinaria, Universidad Distrital
+Estudios de maestría en Estudios Políticos, Universidad Nacional de Colombia</t>
+        </is>
+      </c>
+      <c r="AE6" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Se ha destacado por ocupar cargos de liderazgo en el sector educativo nacional y distrital
+Lideró proyectos estratégicos para fortalecer el acceso y la cobertura de la educación superior
+Consultor del PNUD y participante en la formulación de políticas de educación y paz en Colombia</t>
+        </is>
+      </c>
     </row>
-    <row r="7" spans="1:28" ht="58" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" ht="58" x14ac:dyDescent="0.35">
       <c r="A7" s="64">
         <v>6</v>
       </c>
@@ -3065,8 +3151,11 @@
       <c r="AB7" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC7" s="69"/>
+      <c r="AD7" s="69"/>
+      <c r="AE7" s="69"/>
     </row>
-    <row r="8" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="64">
         <v>7</v>
       </c>
@@ -3147,8 +3236,27 @@
       <c r="AB8" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC8" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Director Colombia, IXL Center</t>
+        </is>
+      </c>
+      <c r="AD8" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MBA, Hult International Business School
+No Code AI and Machine Learning: Building Data Science Solutions, MIT Professional Education</t>
+        </is>
+      </c>
+      <c r="AE8" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Responsable de la implementación de sistemas de innovación en más de 800 empresas alrededor del mundo, con crecimiento y opciones estratégicas en Colombia, Guatemala, Honduras, México y España
+En el Innovation Management Institute ha impartido cursos de formación y certificación en innovación a más de 2.000 personas en todo el mundo
+Entrenador, mentor y facilitador de más de 300 equipos a nivel global
+Capacitó y educó a más de 2.000 personas en sistemas de gestión de innovación con enfoque en resultados económicos</t>
+        </is>
+      </c>
     </row>
-    <row r="9" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:31" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="64">
         <v>8</v>
       </c>
@@ -3229,8 +3337,26 @@
       <c r="AB9" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC9" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Investigadora y Profesora Titular, Universidad de La Sabana</t>
+        </is>
+      </c>
+      <c r="AD9" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingeniera de Alimentos
+Doctorado en Ciencia y Tecnología de Alimentos, Universidad Politécnica de Valencia</t>
+        </is>
+      </c>
+      <c r="AE9" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Más de 20 años de experiencia en docencia, investigación y gestión académica en educación superior
+Directora General de Investigación de la Universidad de La Sabana (2021–2025), liderando estrategias de investigación e innovación
+Investigadora Senior reconocida por Minciencias, líder de grupo y autora en ciencia de alimentos y nutrición</t>
+        </is>
+      </c>
     </row>
-    <row r="10" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="64">
         <v>9</v>
       </c>
@@ -3311,8 +3437,29 @@
       <c r="AB10" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC10" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consultor, investigador y experto en políticas educativas</t>
+        </is>
+      </c>
+      <c r="AD10" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Licenciado en Filosofía (Universidad Javeriana)
+Magíster en Economía (Universidad de los Andes)</t>
+        </is>
+      </c>
+      <c r="AE10" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Más de 25 años de experiencia en educación
+Secretario de Educación de Bogotá (2005-2007)
+Exrector de la Universidad Distrital y Universidad CAFAM
+Consultor de UNESCO y Naciones Unidas en América Latina y África
+Miembro permanente de la Academia Colombiana de Pedagogía y Educación
+Actualmente funge como asesor del Ministerio de Educación</t>
+        </is>
+      </c>
     </row>
-    <row r="11" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:31" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A11" s="64">
         <v>10</v>
       </c>
@@ -3393,8 +3540,28 @@
       <c r="AB11" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC11" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vicerrector de Medios y Mediaciones Pedagógicas, UNAD</t>
+        </is>
+      </c>
+      <c r="AD11" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ingeniero Electrónico
+Doctor en Salud Pública
+Máster en Ingeniería Telemática
+Especialista en Gestión de la Innovación Tecnológica</t>
+        </is>
+      </c>
+      <c r="AE11" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Más de 20 años de experiencia en investigación, innovación, transformación digital y educación superior
+Vicerrector de Medios y Mediaciones Pedagógicas de la UNAD desde 2015, impulsando ecosistemas de aprendizaje digital e innovación educativa
+Líder en transformación digital, innovación educativa e inteligencia artificial aplicada a la educación</t>
+        </is>
+      </c>
     </row>
-    <row r="12" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="64">
         <v>11</v>
       </c>
@@ -3475,8 +3642,26 @@
       <c r="AB12" s="66" t="b">
         <v>1</v>
       </c>
+      <c r="AC12" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vicerrector de Servicios a Aspirantes, Estudiantes y Egresados, UNAD</t>
+        </is>
+      </c>
+      <c r="AD12" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Doctor en Educación a Distancia y Tecnología Instruccional</t>
+        </is>
+      </c>
+      <c r="AE12" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Representante del Comité Asesor ante el Consejo Nacional de Rectores del SUE
+Líder con amplia trayectoria en gestión y dirección universitaria en la UNAD
+Experiencia en cargos directivos como Vicerrector, Decano y Director de Planeación
+Autor de publicaciones sobre educación a distancia, calidad educativa y efectividad organizacional</t>
+        </is>
+      </c>
     </row>
-    <row r="13" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A13" s="64">
         <v>12</v>
       </c>
@@ -3486,8 +3671,10 @@
       <c r="C13" s="67" t="s">
         <v>160</v>
       </c>
-      <c r="D13" s="67" t="s">
-        <v>15</v>
+      <c r="D13" s="67" t="inlineStr">
+        <is>
+          <t>Ana Lucía Chávez Correal</t>
+        </is>
       </c>
       <c r="E13" s="67" t="s">
         <v>168</v>
@@ -3520,11 +3707,15 @@
       <c r="O13" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="P13" s="69" t="s">
-        <v>149</v>
-      </c>
-      <c r="Q13" s="69" t="s">
-        <v>15</v>
+      <c r="P13" s="69" t="inlineStr">
+        <is>
+          <t>ana-lucia-chavez-correal</t>
+        </is>
+      </c>
+      <c r="Q13" s="69" t="inlineStr">
+        <is>
+          <t>Ana Lucía Chávez Correal</t>
+        </is>
       </c>
       <c r="R13" s="69" t="s">
         <v>143</v>
@@ -3556,6 +3747,26 @@
       </c>
       <c r="AB13" s="66" t="b">
         <v>1</v>
+      </c>
+      <c r="AC13" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Integrante del equipo académico del Programa Retos – ASCUN</t>
+        </is>
+      </c>
+      <c r="AD13" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Psicóloga, Universidad Católica de Colombia
+Magíster en Dirección Universitaria, Universidad de los Andes
+Especialista en Docencia Universitaria</t>
+        </is>
+      </c>
+      <c r="AE13" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Integrante del equipo académico-técnico de ASCUN y coordinadora académica del Programa Retos
+Amplia experiencia en dirección, planeación y gestión académica en educación superior
+Liderazgo en desarrollo curricular, calidad institucional y procesos de acreditación
+Participación en iniciativas nacionales de política educativa, incluyendo la Comisión Gestora del Plan Nacional Decenal de Educación 2016–2026</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: sincroniza correcciones del Excel y mejora la lista de conferencistas
Actualiza el Excel en uso con las correcciones del archivo maestro
(ciudad de la jornada de apertura corregida a Soacha, texto alternativo
de Ana Lucía Chávez Correal) preservando las columnas de perfil
extendido y las imágenes de la hoja Encuentros Realizados.

En la lista de conferencistas: se integra la columna "jornada" como
dato principal de cada fila, se colapsa por defecto en un panel
desplegable, y se renombra a "Lista de conferencistas".
</commit_message>
<xml_diff>
--- a/portal-web/data/source-conferencistas/Participacion jornadas.xlsx
+++ b/portal-web/data/source-conferencistas/Participacion jornadas.xlsx
@@ -2624,8 +2624,10 @@
       <c r="D2" s="67" t="s">
         <v>95</v>
       </c>
-      <c r="E2" s="67" t="s">
-        <v>161</v>
+      <c r="E2" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 de marzo - Soacha</t>
+        </is>
       </c>
       <c r="F2" s="67">
         <v>3</v>
@@ -2633,8 +2635,10 @@
       <c r="G2" s="67">
         <v>4</v>
       </c>
-      <c r="H2" s="67" t="s">
-        <v>98</v>
+      <c r="H2" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Soacha</t>
+        </is>
       </c>
       <c r="I2" s="67"/>
       <c r="J2" s="67">
@@ -2661,14 +2665,18 @@
       <c r="S2" s="69" t="s">
         <v>97</v>
       </c>
-      <c r="T2" s="69" t="s">
-        <v>98</v>
+      <c r="T2" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Soacha</t>
+        </is>
       </c>
       <c r="U2" s="69" t="s">
         <v>99</v>
       </c>
-      <c r="V2" s="69" t="s">
-        <v>100</v>
+      <c r="V2" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Jornada de apertura realizada en Soacha con la participación del Grupo Estratégico.</t>
+        </is>
       </c>
       <c r="W2" s="69"/>
       <c r="X2" s="69"/>
@@ -2978,8 +2986,10 @@
       <c r="D6" s="67" t="s">
         <v>76</v>
       </c>
-      <c r="E6" s="67" t="s">
-        <v>165</v>
+      <c r="E6" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13 de mayo - Chía</t>
+        </is>
       </c>
       <c r="F6" s="67">
         <v>5</v>
@@ -3081,8 +3091,10 @@
       <c r="D7" s="67" t="s">
         <v>126</v>
       </c>
-      <c r="E7" s="67" t="s">
-        <v>165</v>
+      <c r="E7" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13 de mayo - Chía</t>
+        </is>
       </c>
       <c r="F7" s="67">
         <v>5</v>
@@ -3491,8 +3503,10 @@
       <c r="K11" s="67">
         <v>515</v>
       </c>
-      <c r="L11" s="67" t="s">
-        <v>81</v>
+      <c r="L11" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conversatorio con vicerrectores de la UNAD y conferencia de la Dra. Ana Lucía Chávez Correal.</t>
+        </is>
       </c>
       <c r="M11" s="67" t="s">
         <v>46</v>
@@ -3593,8 +3607,10 @@
       <c r="K12" s="67">
         <v>515</v>
       </c>
-      <c r="L12" s="67" t="s">
-        <v>81</v>
+      <c r="L12" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conversatorio con vicerrectores de la UNAD y conferencia de la Dra. Ana Lucía Chávez Correal.</t>
+        </is>
       </c>
       <c r="M12" s="67" t="s">
         <v>46</v>
@@ -3695,8 +3711,10 @@
       <c r="K13" s="67">
         <v>515</v>
       </c>
-      <c r="L13" s="67" t="s">
-        <v>81</v>
+      <c r="L13" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Conversatorio con vicerrectores de la UNAD y conferencia de la Dra. Ana Lucía Chávez Correal.</t>
+        </is>
       </c>
       <c r="M13" s="67" t="s">
         <v>46</v>
@@ -3736,8 +3754,10 @@
         <v>46</v>
       </c>
       <c r="X13" s="69"/>
-      <c r="Y13" s="69" t="s">
-        <v>151</v>
+      <c r="Y13" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fotografía de Ana Lucía Chávez Correal</t>
+        </is>
       </c>
       <c r="Z13" s="66">
         <v>12</v>

</xml_diff>

<commit_message>
fix: quita la hora de la fecha mostrada para Ricardo Moreno Patiño
El campo fecha_card de su fila incluía "13 de mayo, 8:30 a. m."; se
deja solo "13 de mayo" para que la card y la lista de conferencistas
muestren la fecha sin hora, igual que el resto de los registros.
</commit_message>
<xml_diff>
--- a/portal-web/data/source-conferencistas/Participacion jornadas.xlsx
+++ b/portal-web/data/source-conferencistas/Participacion jornadas.xlsx
@@ -3030,8 +3030,10 @@
       <c r="R6" s="69" t="s">
         <v>121</v>
       </c>
-      <c r="S6" s="69" t="s">
-        <v>122</v>
+      <c r="S6" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13 de mayo</t>
+        </is>
       </c>
       <c r="T6" s="69" t="s">
         <v>98</v>

</xml_diff>

<commit_message>
fix: usa los nombres completos del Excel y completa el perfil de Martha Duque
Corrige "Leonardo Yunda" -> "Leonardo Emilio Yunda Perlaza" e "Indira
Sotelo" -> "Luz Indira Sotelo Díaz" en la hoja Base de Datos (nombre_card,
participante, texto alternativo) y en las etiquetas de comentarios
compartidos de Valoraciones, para que coincidan con el nombre completo
registrado en la hoja Encuentros Realizados del mismo Excel.

Reemplaza la foto de la jornada de apertura por la imagen de Soacha
(la sede real del evento, ya corregida en el Excel). Completa la fila
de Martha Lucía Duque Ramírez con foto, cargo, formación académica y
trayectoria destacada extraídos de su perfil en PPTX.
</commit_message>
<xml_diff>
--- a/portal-web/data/source-conferencistas/Participacion jornadas.xlsx
+++ b/portal-web/data/source-conferencistas/Participacion jornadas.xlsx
@@ -3165,9 +3165,25 @@
       <c r="AB7" s="66" t="b">
         <v>1</v>
       </c>
-      <c r="AC7" s="69"/>
-      <c r="AD7" s="69"/>
-      <c r="AE7" s="69"/>
+      <c r="AC7" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Asesora de Aseguramiento de la Calidad de la Educación Superior, Universidad de Cundinamarca</t>
+        </is>
+      </c>
+      <c r="AD7" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Licenciada en Biología y Química
+Magíster en Educación de Adultos
+Doctora en Educación</t>
+        </is>
+      </c>
+      <c r="AE7" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Más de 20 años de experiencia en cargos académicos y administrativos en distintas universidades colombianas
+Participación en procesos de calidad y mejora continua en instituciones de educación superior
+Par académica y asesora, fortaleciendo políticas y procesos educativos en universidades del país</t>
+        </is>
+      </c>
     </row>
     <row r="8" spans="1:31" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="64">
@@ -3280,8 +3296,10 @@
       <c r="C9" s="67" t="s">
         <v>159</v>
       </c>
-      <c r="D9" s="67" t="s">
-        <v>10</v>
+      <c r="D9" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luz Indira Sotelo Díaz</t>
+        </is>
       </c>
       <c r="E9" s="67" t="s">
         <v>166</v>
@@ -3317,8 +3335,10 @@
       <c r="P9" s="69" t="s">
         <v>136</v>
       </c>
-      <c r="Q9" s="69" t="s">
-        <v>10</v>
+      <c r="Q9" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Luz Indira Sotelo Díaz</t>
+        </is>
       </c>
       <c r="R9" s="69" t="s">
         <v>132</v>
@@ -3339,8 +3359,10 @@
         <v>41</v>
       </c>
       <c r="X9" s="69"/>
-      <c r="Y9" s="69" t="s">
-        <v>137</v>
+      <c r="Y9" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fotografía de Luz Indira Sotelo Díaz</t>
+        </is>
       </c>
       <c r="Z9" s="66">
         <v>8</v>
@@ -3483,8 +3505,10 @@
       <c r="C11" s="67" t="s">
         <v>160</v>
       </c>
-      <c r="D11" s="67" t="s">
-        <v>13</v>
+      <c r="D11" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leonardo Emilio Yunda Perlaza</t>
+        </is>
       </c>
       <c r="E11" s="67" t="s">
         <v>168</v>
@@ -3522,8 +3546,10 @@
       <c r="P11" s="69" t="s">
         <v>142</v>
       </c>
-      <c r="Q11" s="69" t="s">
-        <v>13</v>
+      <c r="Q11" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leonardo Emilio Yunda Perlaza</t>
+        </is>
       </c>
       <c r="R11" s="69" t="s">
         <v>143</v>
@@ -3544,8 +3570,10 @@
         <v>46</v>
       </c>
       <c r="X11" s="69"/>
-      <c r="Y11" s="69" t="s">
-        <v>146</v>
+      <c r="Y11" s="69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fotografía de Leonardo Emilio Yunda Perlaza</t>
+        </is>
       </c>
       <c r="Z11" s="66">
         <v>10</v>

</xml_diff>